<commit_message>
chore: update trackers with gap-closing work from Session 7b
Added items 7-9 to ACTION-TRACKER: API smoke test results, outcomes
query fixes (visitors_connected 0→8, fit_scores 1→9, navigation 0→27),
and visual CSS fixes applied across 8 pages. Updated MASTER-ACTION-PLAN
notes for rows 36/70/72 to reflect verified-complete status.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MASTER-ACTION-PLAN.xlsx
+++ b/MASTER-ACTION-PLAN.xlsx
@@ -1917,7 +1917,7 @@
       </c>
       <c r="H36" s="21" t="inlineStr">
         <is>
-          <t>Done — Full audit of 10 pages against VISUAL-STANDARDS.md. Report at docs/VISUAL-AUDIT-REPORT.md. Session 7b.</t>
+          <t>Done — Audit report at docs/VISUAL-AUDIT-REPORT.md. CSS fixes applied: hardcoded colors replaced in 3 pages, light mode overrides added to all 8 pages with inline styles, grid gaps standardized to 24px across 4 pages, index.html font loading trimmed from 11 to 1 family. Session 7b.</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="H70" s="21" t="inlineStr">
         <is>
-          <t>Done — GET /api/fenix/outcomes endpoint added. Aggregates conversations, visitors, connections, fit scores, navigation. Session 7b.</t>
+          <t>Done — GET /api/fenix/outcomes added and query-validated. Queries visitor_connects for connections (8), case-insensitive fit score search (9), page path navigation (27). Engagement rate uses batch query. Session 7b.</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="H72" s="21" t="inlineStr">
         <is>
-          <t>Done — Full CRUD API, 32 initiatives migrated from career-highlights.html, domain/company filtering. Session 7b.</t>
+          <t>Done — Full CRUD API, 32 initiatives migrated, all 8 endpoints smoke-tested live against cc.kiranrao.ai. Filtering by domain/company/era/search verified. Session 7b.</t>
         </is>
       </c>
     </row>
@@ -4309,12 +4309,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4437,21 +4437,21 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>Session 7b (Apr 12, 2026)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>6 Claude items completed: career-initiatives entity, outcomes endpoint,</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>learning page, bento dimensions, visual audit, add-skills confirmation</t>
         </is>

</xml_diff>

<commit_message>
feat: complete 20 Claude-only zero-dependency items (Session 7c)
Blog: rename ca192ebf → invisible-rail-ach-payments, add to hub, 301 redirect
Docs: triptych in INDEX-HOMEPAGE, DIA Fund templates, contrast audit, now-page
      assessment, awards research, CC auto-now spec, teardown accuracy audit,
      card redesign spec, picker bypass verification, Scannibal disclaimers
Teardowns: add last-updated dates to 6 detail pages
Blog: generate OG cards for 2 posts, update meta tags
V6: add incremental MJ generation workflow with 14 ready-to-use prompts
CC: add action item reconciliation script (reconcile_action_items.py)
Trackers: update ACTION-TRACKER.md and MASTER-ACTION-PLAN.xlsx

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MASTER-ACTION-PLAN.xlsx
+++ b/MASTER-ACTION-PLAN.xlsx
@@ -4173,7 +4173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="15" min="1" max="1"/>
@@ -4454,6 +4454,55 @@
       <c r="A35" s="15" t="inlineStr">
         <is>
           <t>learning page, bento dimensions, visual audit, add-skills confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Session 7c (Apr 12, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20 Claude-only zero-dependency items completed from ACTION-TRACKER:</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Blog URL rework, triptych docs, DIA Fund templates, contrast audit,</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>teardown dates, OG cards, Scannibal disclaimers, V6 prompt update,</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>card redesign spec, /Now assessment, awards research, CC auto-now spec,</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>reconciliation script, teardown accuracy audit, picker bypass verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Note: These items are from ACTION-TRACKER.md (221 items), not this Excel (79 items).</t>
         </is>
       </c>
     </row>

</xml_diff>